<commit_message>
Drop the public (no sign-in) route and pilot task 6
SFPUC's portal doesn't allow anonymous access. Remove the public view,
the no-sign-in tests and the Survey123-only no-account pilot task, and
rebalance the team criteria weights.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WcX7gz835Uu2NoHiASCWjE
</commit_message>
<xml_diff>
--- a/docs/kit/pilot/pilot-scorecard.xlsx
+++ b/docs/kit/pilot/pilot-scorecard.xlsx
@@ -688,7 +688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:X13"/>
+  <dimension ref="A1:X11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1847,234 +1847,6 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="15" t="inlineStr">
-        <is>
-          <t>T6</t>
-        </is>
-      </c>
-      <c r="B12" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C12" s="15" t="inlineStr">
-        <is>
-          <t>3803</t>
-        </is>
-      </c>
-      <c r="D12" s="15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E12" s="15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F12" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G12" s="15" t="n">
-        <v>55</v>
-      </c>
-      <c r="H12" s="15" t="n">
-        <v>50</v>
-      </c>
-      <c r="I12" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J12" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" s="15" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="L12" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M12" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N12" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O12" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="P12" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Q12" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="R12" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="S12" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="T12" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U12" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="V12" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W12" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="X12" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="15" t="inlineStr">
-        <is>
-          <t>T6</t>
-        </is>
-      </c>
-      <c r="B13" s="15" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="C13" s="15" t="inlineStr">
-        <is>
-          <t>3808</t>
-        </is>
-      </c>
-      <c r="D13" s="15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E13" s="15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F13" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G13" s="15" t="n">
-        <v>54</v>
-      </c>
-      <c r="H13" s="15" t="n">
-        <v>50</v>
-      </c>
-      <c r="I13" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J13" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" s="15" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="L13" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M13" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N13" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O13" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="P13" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Q13" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="R13" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="S13" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="T13" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U13" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="V13" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W13" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="X13" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -2087,7 +1859,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -2142,11 +1914,11 @@
         </is>
       </c>
       <c r="B5" s="8">
-        <f>COUNTIFS(Tasks!$C$2:$C$89,B$3,Tasks!$E$2:$E$89,"&lt;&gt;T6",Tasks!$I$2:$I$89,"&lt;&gt;")</f>
+        <f>COUNTIFS(Tasks!$C$2:$C$81,B$3,Tasks!$I$2:$I$81,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>COUNTIFS(Tasks!$C$2:$C$89,C$3,Tasks!$E$2:$E$89,"&lt;&gt;T6",Tasks!$I$2:$I$89,"&lt;&gt;")</f>
+        <f>COUNTIFS(Tasks!$C$2:$C$81,C$3,Tasks!$I$2:$I$81,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="D5" s="8" t="inlineStr">
@@ -2162,11 +1934,11 @@
         </is>
       </c>
       <c r="B6" s="9">
-        <f>IFERROR(COUNTIFS(Tasks!$C$2:$C$89,B$3,Tasks!$E$2:$E$89,"&lt;&gt;T6",Tasks!$I$2:$I$89,"Alone")/B5,"")</f>
+        <f>IFERROR(COUNTIFS(Tasks!$C$2:$C$81,B$3,Tasks!$I$2:$I$81,"Alone")/B5,"")</f>
         <v/>
       </c>
       <c r="C6" s="9">
-        <f>IFERROR(COUNTIFS(Tasks!$C$2:$C$89,C$3,Tasks!$E$2:$E$89,"&lt;&gt;T6",Tasks!$I$2:$I$89,"Alone")/C5,"")</f>
+        <f>IFERROR(COUNTIFS(Tasks!$C$2:$C$81,C$3,Tasks!$I$2:$I$81,"Alone")/C5,"")</f>
         <v/>
       </c>
       <c r="D6" s="8" t="inlineStr">
@@ -2182,11 +1954,11 @@
         </is>
       </c>
       <c r="B7" s="9">
-        <f>IFERROR(COUNTIFS(Tasks!$C$2:$C$89,B$3,Tasks!$E$2:$E$89,"&lt;&gt;T6",Tasks!$I$2:$I$89,"With help")/B5,"")</f>
+        <f>IFERROR(COUNTIFS(Tasks!$C$2:$C$81,B$3,Tasks!$I$2:$I$81,"With help")/B5,"")</f>
         <v/>
       </c>
       <c r="C7" s="9">
-        <f>IFERROR(COUNTIFS(Tasks!$C$2:$C$89,C$3,Tasks!$E$2:$E$89,"&lt;&gt;T6",Tasks!$I$2:$I$89,"With help")/C5,"")</f>
+        <f>IFERROR(COUNTIFS(Tasks!$C$2:$C$81,C$3,Tasks!$I$2:$I$81,"With help")/C5,"")</f>
         <v/>
       </c>
       <c r="D7" s="8" t="inlineStr"/>
@@ -2198,11 +1970,11 @@
         </is>
       </c>
       <c r="B8" s="9">
-        <f>IFERROR((COUNTIFS(Tasks!$C$2:$C$89,B$3,Tasks!$E$2:$E$89,"&lt;&gt;T6",Tasks!$I$2:$I$89,"Failed")+COUNTIFS(Tasks!$C$2:$C$89,B$3,Tasks!$E$2:$E$89,"&lt;&gt;T6",Tasks!$I$2:$I$89,"Skipped"))/B5,"")</f>
+        <f>IFERROR((COUNTIFS(Tasks!$C$2:$C$81,B$3,Tasks!$I$2:$I$81,"Failed")+COUNTIFS(Tasks!$C$2:$C$81,B$3,Tasks!$I$2:$I$81,"Skipped"))/B5,"")</f>
         <v/>
       </c>
       <c r="C8" s="9">
-        <f>IFERROR((COUNTIFS(Tasks!$C$2:$C$89,C$3,Tasks!$E$2:$E$89,"&lt;&gt;T6",Tasks!$I$2:$I$89,"Failed")+COUNTIFS(Tasks!$C$2:$C$89,C$3,Tasks!$E$2:$E$89,"&lt;&gt;T6",Tasks!$I$2:$I$89,"Skipped"))/C5,"")</f>
+        <f>IFERROR((COUNTIFS(Tasks!$C$2:$C$81,C$3,Tasks!$I$2:$I$81,"Failed")+COUNTIFS(Tasks!$C$2:$C$81,C$3,Tasks!$I$2:$I$81,"Skipped"))/C5,"")</f>
         <v/>
       </c>
       <c r="D8" s="8" t="inlineStr"/>
@@ -2214,11 +1986,11 @@
         </is>
       </c>
       <c r="B9" s="10">
-        <f>IFERROR(AVERAGEIFS(Tasks!$H$2:$H$89,Tasks!$C$2:$C$89,B$3,Tasks!$E$2:$E$89,"&lt;&gt;T6"),"")</f>
+        <f>IFERROR(AVERAGEIFS(Tasks!$H$2:$H$81,Tasks!$C$2:$C$81,B$3),"")</f>
         <v/>
       </c>
       <c r="C9" s="10">
-        <f>IFERROR(AVERAGEIFS(Tasks!$H$2:$H$89,Tasks!$C$2:$C$89,C$3,Tasks!$E$2:$E$89,"&lt;&gt;T6"),"")</f>
+        <f>IFERROR(AVERAGEIFS(Tasks!$H$2:$H$81,Tasks!$C$2:$C$81,C$3),"")</f>
         <v/>
       </c>
       <c r="D9" s="8" t="inlineStr"/>
@@ -2230,11 +2002,11 @@
         </is>
       </c>
       <c r="B10" s="10">
-        <f>IFERROR(AVERAGEIFS(Tasks!$J$2:$J$89,Tasks!$C$2:$C$89,B$3,Tasks!$E$2:$E$89,"&lt;&gt;T6"),"")</f>
+        <f>IFERROR(AVERAGEIFS(Tasks!$J$2:$J$81,Tasks!$C$2:$C$81,B$3),"")</f>
         <v/>
       </c>
       <c r="C10" s="10">
-        <f>IFERROR(AVERAGEIFS(Tasks!$J$2:$J$89,Tasks!$C$2:$C$89,C$3,Tasks!$E$2:$E$89,"&lt;&gt;T6"),"")</f>
+        <f>IFERROR(AVERAGEIFS(Tasks!$J$2:$J$81,Tasks!$C$2:$C$81,C$3),"")</f>
         <v/>
       </c>
       <c r="D10" s="8" t="inlineStr">
@@ -2250,11 +2022,11 @@
         </is>
       </c>
       <c r="B11" s="9">
-        <f>IFERROR((COUNTIFS(Tasks!$C$2:$C$89,B$3,Tasks!$E$2:$E$89,"T5",Tasks!$I$2:$I$89,"Alone")+COUNTIFS(Tasks!$C$2:$C$89,B$3,Tasks!$E$2:$E$89,"T5",Tasks!$I$2:$I$89,"With help"))/COUNTIFS(Tasks!$C$2:$C$89,B$3,Tasks!$E$2:$E$89,"T5",Tasks!$I$2:$I$89,"&lt;&gt;"),"")</f>
+        <f>IFERROR((COUNTIFS(Tasks!$C$2:$C$81,B$3,Tasks!$E$2:$E$81,"T5",Tasks!$I$2:$I$81,"Alone")+COUNTIFS(Tasks!$C$2:$C$81,B$3,Tasks!$E$2:$E$81,"T5",Tasks!$I$2:$I$81,"With help"))/COUNTIFS(Tasks!$C$2:$C$81,B$3,Tasks!$E$2:$E$81,"T5",Tasks!$I$2:$I$81,"&lt;&gt;"),"")</f>
         <v/>
       </c>
       <c r="C11" s="9">
-        <f>IFERROR((COUNTIFS(Tasks!$C$2:$C$89,C$3,Tasks!$E$2:$E$89,"T5",Tasks!$I$2:$I$89,"Alone")+COUNTIFS(Tasks!$C$2:$C$89,C$3,Tasks!$E$2:$E$89,"T5",Tasks!$I$2:$I$89,"With help"))/COUNTIFS(Tasks!$C$2:$C$89,C$3,Tasks!$E$2:$E$89,"T5",Tasks!$I$2:$I$89,"&lt;&gt;"),"")</f>
+        <f>IFERROR((COUNTIFS(Tasks!$C$2:$C$81,C$3,Tasks!$E$2:$E$81,"T5",Tasks!$I$2:$I$81,"Alone")+COUNTIFS(Tasks!$C$2:$C$81,C$3,Tasks!$E$2:$E$81,"T5",Tasks!$I$2:$I$81,"With help"))/COUNTIFS(Tasks!$C$2:$C$81,C$3,Tasks!$E$2:$E$81,"T5",Tasks!$I$2:$I$81,"&lt;&gt;"),"")</f>
         <v/>
       </c>
       <c r="D11" s="8" t="inlineStr">
@@ -2320,11 +2092,11 @@
         </is>
       </c>
       <c r="B15" s="8">
-        <f>COUNTIFS('Data check'!$D$2:$D$109,B$3,'Data check'!$B$2:$B$109,"&lt;&gt;T6",'Data check'!$G$2:$G$109,"&gt;=0")</f>
+        <f>COUNTIFS('Data check'!$D$2:$D$109,B$3,'Data check'!$G$2:$G$109,"&gt;=0")</f>
         <v/>
       </c>
       <c r="C15" s="8">
-        <f>COUNTIFS('Data check'!$D$2:$D$109,C$3,'Data check'!$B$2:$B$109,"&lt;&gt;T6",'Data check'!$G$2:$G$109,"&gt;=0")</f>
+        <f>COUNTIFS('Data check'!$D$2:$D$109,C$3,'Data check'!$G$2:$G$109,"&gt;=0")</f>
         <v/>
       </c>
       <c r="D15" s="8" t="inlineStr">
@@ -2340,11 +2112,11 @@
         </is>
       </c>
       <c r="B16" s="9">
-        <f>IFERROR(COUNTIFS('Data check'!$D$2:$D$109,B$3,'Data check'!$B$2:$B$109,"&lt;&gt;T6",'Data check'!$F$2:$F$109,"Yes")/B15,"")</f>
+        <f>IFERROR(COUNTIFS('Data check'!$D$2:$D$109,B$3,'Data check'!$F$2:$F$109,"Yes")/B15,"")</f>
         <v/>
       </c>
       <c r="C16" s="9">
-        <f>IFERROR(COUNTIFS('Data check'!$D$2:$D$109,C$3,'Data check'!$B$2:$B$109,"&lt;&gt;T6",'Data check'!$F$2:$F$109,"Yes")/C15,"")</f>
+        <f>IFERROR(COUNTIFS('Data check'!$D$2:$D$109,C$3,'Data check'!$F$2:$F$109,"Yes")/C15,"")</f>
         <v/>
       </c>
       <c r="D16" s="8" t="inlineStr"/>
@@ -2356,11 +2128,11 @@
         </is>
       </c>
       <c r="B17" s="9">
-        <f>IFERROR(COUNTIFS('Data check'!$D$2:$D$109,B$3,'Data check'!$B$2:$B$109,"&lt;&gt;T6",'Data check'!$G$2:$G$109,0)/B15,"")</f>
+        <f>IFERROR(COUNTIFS('Data check'!$D$2:$D$109,B$3,'Data check'!$G$2:$G$109,0)/B15,"")</f>
         <v/>
       </c>
       <c r="C17" s="9">
-        <f>IFERROR(COUNTIFS('Data check'!$D$2:$D$109,C$3,'Data check'!$B$2:$B$109,"&lt;&gt;T6",'Data check'!$G$2:$G$109,0)/C15,"")</f>
+        <f>IFERROR(COUNTIFS('Data check'!$D$2:$D$109,C$3,'Data check'!$G$2:$G$109,0)/C15,"")</f>
         <v/>
       </c>
       <c r="D17" s="8" t="inlineStr"/>
@@ -2372,11 +2144,11 @@
         </is>
       </c>
       <c r="B18" s="10">
-        <f>IFERROR(AVERAGEIFS('Data check'!$G$2:$G$109,'Data check'!$D$2:$D$109,B$3,'Data check'!$B$2:$B$109,"&lt;&gt;T6"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Data check'!$G$2:$G$109,'Data check'!$D$2:$D$109,B$3),"")</f>
         <v/>
       </c>
       <c r="C18" s="10">
-        <f>IFERROR(AVERAGEIFS('Data check'!$G$2:$G$109,'Data check'!$D$2:$D$109,C$3,'Data check'!$B$2:$B$109,"&lt;&gt;T6"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Data check'!$G$2:$G$109,'Data check'!$D$2:$D$109,C$3),"")</f>
         <v/>
       </c>
       <c r="D18" s="8" t="inlineStr"/>
@@ -2384,7 +2156,7 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>No-account test (task 6, Survey123 only)</t>
+          <t>Must pass</t>
         </is>
       </c>
       <c r="B19" s="7" t="n"/>
@@ -2394,195 +2166,143 @@
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>Task 6 done alone</t>
-        </is>
-      </c>
-      <c r="B20" s="9" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="C20" s="9">
-        <f>IFERROR(COUNTIFS(Tasks!$E$2:$E$89,"T6",Tasks!$I$2:$I$89,"Alone")/COUNTIFS(Tasks!$E$2:$E$89,"T6",Tasks!$I$2:$I$89,"&lt;&gt;"),"")</f>
+          <t>80% or more done alone</t>
+        </is>
+      </c>
+      <c r="B20" s="8">
+        <f>IF(B6="","",IF(B6&gt;=0.8,"PASS","FAIL"))</f>
         <v/>
       </c>
-      <c r="D20" s="8" t="n"/>
+      <c r="C20" s="8">
+        <f>IF(C6="","",IF(C6&gt;=0.8,"PASS","FAIL"))</f>
+        <v/>
+      </c>
+      <c r="D20" s="8" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>Task 6 records tied to a hydrant</t>
-        </is>
-      </c>
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="C21" s="9">
-        <f>IFERROR(COUNTIFS('Data check'!$B$2:$B$109,"T6",'Data check'!$F$2:$F$109,"Yes")/COUNTIFS('Data check'!$B$2:$B$109,"T6",'Data check'!$G$2:$G$109,"&gt;=0"),"")</f>
+          <t>95% or more tied to the right hydrant</t>
+        </is>
+      </c>
+      <c r="B21" s="8">
+        <f>IF(B16="","",IF(B16&gt;=0.95,"PASS","FAIL"))</f>
         <v/>
       </c>
-      <c r="D21" s="8" t="n"/>
+      <c r="C21" s="8">
+        <f>IF(C16="","",IF(C16&gt;=0.95,"PASS","FAIL"))</f>
+        <v/>
+      </c>
+      <c r="D21" s="8" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>Must pass</t>
-        </is>
-      </c>
-      <c r="B22" s="7" t="n"/>
-      <c r="C22" s="7" t="n"/>
-      <c r="D22" s="7" t="n"/>
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Offline synced for every tester</t>
+        </is>
+      </c>
+      <c r="B22" s="8">
+        <f>IF(B11="","",IF(B11=1,"PASS","FAIL"))</f>
+        <v/>
+      </c>
+      <c r="C22" s="8">
+        <f>IF(C11="","",IF(C11=1,"PASS","FAIL"))</f>
+        <v/>
+      </c>
+      <c r="D22" s="8" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="inlineStr">
-        <is>
-          <t>80% or more done alone</t>
-        </is>
-      </c>
-      <c r="B23" s="8">
-        <f>IF(B6="","",IF(B6&gt;=0.8,"PASS","FAIL"))</f>
-        <v/>
-      </c>
-      <c r="C23" s="8">
-        <f>IF(C6="","",IF(C6&gt;=0.8,"PASS","FAIL"))</f>
-        <v/>
-      </c>
-      <c r="D23" s="8" t="inlineStr"/>
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Scores (out of 100)</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="n"/>
+      <c r="C23" s="7" t="n"/>
+      <c r="D23" s="7" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>95% or more tied to the right hydrant</t>
-        </is>
-      </c>
-      <c r="B24" s="8">
-        <f>IF(B16="","",IF(B16&gt;=0.95,"PASS","FAIL"))</f>
+          <t>Crew score</t>
+        </is>
+      </c>
+      <c r="B24" s="11">
+        <f>IFERROR(100*(0.4*B6+0.3*(B10-1)/6+0.3*(B12-1)/4),"")</f>
         <v/>
       </c>
-      <c r="C24" s="8">
-        <f>IF(C16="","",IF(C16&gt;=0.95,"PASS","FAIL"))</f>
+      <c r="C24" s="11">
+        <f>IFERROR(100*(0.4*C6+0.3*(C10-1)/6+0.3*(C12-1)/4),"")</f>
         <v/>
       </c>
-      <c r="D24" s="8" t="inlineStr"/>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>40% done alone, 30% ease, 30% after-app</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>Offline synced for every tester</t>
-        </is>
-      </c>
-      <c r="B25" s="8">
-        <f>IF(B11="","",IF(B11=1,"PASS","FAIL"))</f>
+          <t>Team score</t>
+        </is>
+      </c>
+      <c r="B25" s="11">
+        <f>IF('Team criteria'!F$9=0,"",100*'Team criteria'!F$9/(5*'Team criteria'!$C$9))</f>
         <v/>
       </c>
-      <c r="C25" s="8">
-        <f>IF(C11="","",IF(C11=1,"PASS","FAIL"))</f>
+      <c r="C25" s="11">
+        <f>IF('Team criteria'!G$9=0,"",100*'Team criteria'!G$9/(5*'Team criteria'!$C$9))</f>
         <v/>
       </c>
-      <c r="D25" s="8" t="inlineStr"/>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Weighted Team criteria</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>Scores (out of 100)</t>
-        </is>
-      </c>
-      <c r="B26" s="7" t="n"/>
-      <c r="C26" s="7" t="n"/>
-      <c r="D26" s="7" t="n"/>
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>Combined score</t>
+        </is>
+      </c>
+      <c r="B26" s="11">
+        <f>IFERROR((B24+B25)/2,"")</f>
+        <v/>
+      </c>
+      <c r="C26" s="11">
+        <f>IFERROR((C24+C25)/2,"")</f>
+        <v/>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>Crew and team weighted equally</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="inlineStr">
-        <is>
-          <t>Crew score</t>
-        </is>
-      </c>
-      <c r="B27" s="11">
-        <f>IFERROR(100*(0.4*B6+0.3*(B10-1)/6+0.3*(B12-1)/4),"")</f>
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>Closer than 10%? (then tester preference decides, see the pilot page)</t>
+        </is>
+      </c>
+      <c r="B27" s="13">
+        <f>IFERROR(IF(ABS(B26-C26)&lt;0.1*MAX(B26,C26),"Yes","No"),"")</f>
         <v/>
       </c>
-      <c r="C27" s="11">
-        <f>IFERROR(100*(0.4*C6+0.3*(C10-1)/6+0.3*(C12-1)/4),"")</f>
-        <v/>
-      </c>
-      <c r="D27" s="8" t="inlineStr">
-        <is>
-          <t>40% done alone, 30% ease, 30% after-app</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="8" t="inlineStr">
-        <is>
-          <t>Team score</t>
-        </is>
-      </c>
-      <c r="B28" s="11">
-        <f>IF('Team criteria'!F$10=0,"",100*'Team criteria'!F$10/(5*'Team criteria'!$C$10))</f>
-        <v/>
-      </c>
-      <c r="C28" s="11">
-        <f>IF('Team criteria'!G$10=0,"",100*'Team criteria'!G$10/(5*'Team criteria'!$C$10))</f>
-        <v/>
-      </c>
-      <c r="D28" s="8" t="inlineStr">
-        <is>
-          <t>Weighted Team criteria</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="8" t="inlineStr">
-        <is>
-          <t>Combined score</t>
-        </is>
-      </c>
-      <c r="B29" s="11">
-        <f>IFERROR((B27+B28)/2,"")</f>
-        <v/>
-      </c>
-      <c r="C29" s="11">
-        <f>IFERROR((C27+C28)/2,"")</f>
-        <v/>
-      </c>
-      <c r="D29" s="8" t="inlineStr">
-        <is>
-          <t>Crew and team weighted equally</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="12" t="inlineStr">
-        <is>
-          <t>Closer than 10%? (then account access decides, see PILOT-SCRIPT.md)</t>
-        </is>
-      </c>
-      <c r="B30" s="13">
-        <f>IFERROR(IF(ABS(B29-C29)&lt;0.1*MAX(B29,C29),"Yes","No"),"")</f>
-        <v/>
-      </c>
-      <c r="C30" s="14" t="n"/>
-      <c r="D30" s="13" t="inlineStr">
+      <c r="C27" s="14" t="n"/>
+      <c r="D27" s="13" t="inlineStr">
         <is>
           <t>Difference under 10% of the higher score</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Task 6 is reported on its own: the no-account path only exists in Survey123, and those records are expected to arrive without a hydrant link.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="A32:D32"/>
+  <mergeCells count="1">
+    <mergeCell ref="B27:C27"/>
   </mergeCells>
-  <conditionalFormatting sqref="B23:C25">
+  <conditionalFormatting sqref="B20:C22">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"PASS"</formula>
     </cfRule>
@@ -2853,7 +2573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L89"/>
+  <dimension ref="A1:L81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3335,11 +3055,11 @@
     <row r="12">
       <c r="A12" s="15" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="B12" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C12" s="15" t="inlineStr">
         <is>
@@ -3348,22 +3068,22 @@
       </c>
       <c r="D12" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E12" s="15" t="inlineStr">
         <is>
-          <t>T6</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="F12" s="15" t="inlineStr">
         <is>
-          <t>No account (Survey123 only)</t>
+          <t>Routine check</t>
         </is>
       </c>
       <c r="G12" s="15" t="inlineStr">
         <is>
-          <t>3808</t>
+          <t>0291</t>
         </is>
       </c>
       <c r="H12" s="18" t="n"/>
@@ -3393,17 +3113,17 @@
       </c>
       <c r="E13" s="15" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="F13" s="15" t="inlineStr">
         <is>
-          <t>Routine check</t>
+          <t>Low pressure, missing cap</t>
         </is>
       </c>
       <c r="G13" s="15" t="inlineStr">
         <is>
-          <t>0291</t>
+          <t>0490</t>
         </is>
       </c>
       <c r="H13" s="18" t="n"/>
@@ -3433,17 +3153,17 @@
       </c>
       <c r="E14" s="15" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="F14" s="15" t="inlineStr">
         <is>
-          <t>Low pressure, missing cap</t>
+          <t>Several problems</t>
         </is>
       </c>
       <c r="G14" s="15" t="inlineStr">
         <is>
-          <t>0490</t>
+          <t>3641</t>
         </is>
       </c>
       <c r="H14" s="18" t="n"/>
@@ -3473,17 +3193,17 @@
       </c>
       <c r="E15" s="15" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T4</t>
         </is>
       </c>
       <c r="F15" s="15" t="inlineStr">
         <is>
-          <t>Several problems</t>
+          <t>Hydrant not there</t>
         </is>
       </c>
       <c r="G15" s="15" t="inlineStr">
         <is>
-          <t>3641</t>
+          <t>0718</t>
         </is>
       </c>
       <c r="H15" s="18" t="n"/>
@@ -3513,17 +3233,17 @@
       </c>
       <c r="E16" s="15" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>T5</t>
         </is>
       </c>
       <c r="F16" s="15" t="inlineStr">
         <is>
-          <t>Hydrant not there</t>
+          <t>No signal (offline)</t>
         </is>
       </c>
       <c r="G16" s="15" t="inlineStr">
         <is>
-          <t>0718</t>
+          <t>3466</t>
         </is>
       </c>
       <c r="H16" s="18" t="n"/>
@@ -3539,31 +3259,31 @@
         </is>
       </c>
       <c r="B17" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C17" s="15" t="inlineStr">
         <is>
-          <t>Survey123</t>
+          <t>Field Maps</t>
         </is>
       </c>
       <c r="D17" s="15" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E17" s="15" t="inlineStr">
         <is>
-          <t>T5</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="F17" s="15" t="inlineStr">
         <is>
-          <t>No signal (offline)</t>
+          <t>Routine check</t>
         </is>
       </c>
       <c r="G17" s="15" t="inlineStr">
         <is>
-          <t>3466</t>
+          <t>0353</t>
         </is>
       </c>
       <c r="H17" s="18" t="n"/>
@@ -3579,31 +3299,31 @@
         </is>
       </c>
       <c r="B18" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C18" s="15" t="inlineStr">
         <is>
-          <t>Survey123</t>
+          <t>Field Maps</t>
         </is>
       </c>
       <c r="D18" s="15" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E18" s="15" t="inlineStr">
         <is>
-          <t>T6</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="F18" s="15" t="inlineStr">
         <is>
-          <t>No account (Survey123 only)</t>
+          <t>Low pressure, missing cap</t>
         </is>
       </c>
       <c r="G18" s="15" t="inlineStr">
         <is>
-          <t>3803</t>
+          <t>0564</t>
         </is>
       </c>
       <c r="H18" s="18" t="n"/>
@@ -3633,17 +3353,17 @@
       </c>
       <c r="E19" s="15" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="F19" s="15" t="inlineStr">
         <is>
-          <t>Routine check</t>
+          <t>Several problems</t>
         </is>
       </c>
       <c r="G19" s="15" t="inlineStr">
         <is>
-          <t>0353</t>
+          <t>3402</t>
         </is>
       </c>
       <c r="H19" s="18" t="n"/>
@@ -3673,17 +3393,17 @@
       </c>
       <c r="E20" s="15" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T4</t>
         </is>
       </c>
       <c r="F20" s="15" t="inlineStr">
         <is>
-          <t>Low pressure, missing cap</t>
+          <t>Hydrant not there</t>
         </is>
       </c>
       <c r="G20" s="15" t="inlineStr">
         <is>
-          <t>0564</t>
+          <t>0570</t>
         </is>
       </c>
       <c r="H20" s="18" t="n"/>
@@ -3713,17 +3433,17 @@
       </c>
       <c r="E21" s="15" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T5</t>
         </is>
       </c>
       <c r="F21" s="15" t="inlineStr">
         <is>
-          <t>Several problems</t>
+          <t>No signal (offline)</t>
         </is>
       </c>
       <c r="G21" s="15" t="inlineStr">
         <is>
-          <t>3402</t>
+          <t>3467</t>
         </is>
       </c>
       <c r="H21" s="18" t="n"/>
@@ -3735,11 +3455,11 @@
     <row r="22">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C22" s="15" t="inlineStr">
         <is>
@@ -3753,17 +3473,17 @@
       </c>
       <c r="E22" s="15" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="F22" s="15" t="inlineStr">
         <is>
-          <t>Hydrant not there</t>
+          <t>Routine check</t>
         </is>
       </c>
       <c r="G22" s="15" t="inlineStr">
         <is>
-          <t>0570</t>
+          <t>0353</t>
         </is>
       </c>
       <c r="H22" s="18" t="n"/>
@@ -3775,11 +3495,11 @@
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C23" s="15" t="inlineStr">
         <is>
@@ -3793,17 +3513,17 @@
       </c>
       <c r="E23" s="15" t="inlineStr">
         <is>
-          <t>T5</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="F23" s="15" t="inlineStr">
         <is>
-          <t>No signal (offline)</t>
+          <t>Low pressure, missing cap</t>
         </is>
       </c>
       <c r="G23" s="15" t="inlineStr">
         <is>
-          <t>3467</t>
+          <t>0564</t>
         </is>
       </c>
       <c r="H23" s="18" t="n"/>
@@ -3833,17 +3553,17 @@
       </c>
       <c r="E24" s="15" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="F24" s="15" t="inlineStr">
         <is>
-          <t>Routine check</t>
+          <t>Several problems</t>
         </is>
       </c>
       <c r="G24" s="15" t="inlineStr">
         <is>
-          <t>0353</t>
+          <t>3402</t>
         </is>
       </c>
       <c r="H24" s="18" t="n"/>
@@ -3873,17 +3593,17 @@
       </c>
       <c r="E25" s="15" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T4</t>
         </is>
       </c>
       <c r="F25" s="15" t="inlineStr">
         <is>
-          <t>Low pressure, missing cap</t>
+          <t>Hydrant not there</t>
         </is>
       </c>
       <c r="G25" s="15" t="inlineStr">
         <is>
-          <t>0564</t>
+          <t>0570</t>
         </is>
       </c>
       <c r="H25" s="18" t="n"/>
@@ -3913,17 +3633,17 @@
       </c>
       <c r="E26" s="15" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T5</t>
         </is>
       </c>
       <c r="F26" s="15" t="inlineStr">
         <is>
-          <t>Several problems</t>
+          <t>No signal (offline)</t>
         </is>
       </c>
       <c r="G26" s="15" t="inlineStr">
         <is>
-          <t>3402</t>
+          <t>3467</t>
         </is>
       </c>
       <c r="H26" s="18" t="n"/>
@@ -3939,31 +3659,31 @@
         </is>
       </c>
       <c r="B27" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C27" s="15" t="inlineStr">
         <is>
-          <t>Field Maps</t>
+          <t>Survey123</t>
         </is>
       </c>
       <c r="D27" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E27" s="15" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="F27" s="15" t="inlineStr">
         <is>
-          <t>Hydrant not there</t>
+          <t>Routine check</t>
         </is>
       </c>
       <c r="G27" s="15" t="inlineStr">
         <is>
-          <t>0570</t>
+          <t>0291</t>
         </is>
       </c>
       <c r="H27" s="18" t="n"/>
@@ -3979,31 +3699,31 @@
         </is>
       </c>
       <c r="B28" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C28" s="15" t="inlineStr">
         <is>
-          <t>Field Maps</t>
+          <t>Survey123</t>
         </is>
       </c>
       <c r="D28" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E28" s="15" t="inlineStr">
         <is>
-          <t>T5</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="F28" s="15" t="inlineStr">
         <is>
-          <t>No signal (offline)</t>
+          <t>Low pressure, missing cap</t>
         </is>
       </c>
       <c r="G28" s="15" t="inlineStr">
         <is>
-          <t>3467</t>
+          <t>0490</t>
         </is>
       </c>
       <c r="H28" s="18" t="n"/>
@@ -4033,17 +3753,17 @@
       </c>
       <c r="E29" s="15" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="F29" s="15" t="inlineStr">
         <is>
-          <t>Routine check</t>
+          <t>Several problems</t>
         </is>
       </c>
       <c r="G29" s="15" t="inlineStr">
         <is>
-          <t>0291</t>
+          <t>3641</t>
         </is>
       </c>
       <c r="H29" s="18" t="n"/>
@@ -4073,17 +3793,17 @@
       </c>
       <c r="E30" s="15" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T4</t>
         </is>
       </c>
       <c r="F30" s="15" t="inlineStr">
         <is>
-          <t>Low pressure, missing cap</t>
+          <t>Hydrant not there</t>
         </is>
       </c>
       <c r="G30" s="15" t="inlineStr">
         <is>
-          <t>0490</t>
+          <t>0718</t>
         </is>
       </c>
       <c r="H30" s="18" t="n"/>
@@ -4113,17 +3833,17 @@
       </c>
       <c r="E31" s="15" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T5</t>
         </is>
       </c>
       <c r="F31" s="15" t="inlineStr">
         <is>
-          <t>Several problems</t>
+          <t>No signal (offline)</t>
         </is>
       </c>
       <c r="G31" s="15" t="inlineStr">
         <is>
-          <t>3641</t>
+          <t>3466</t>
         </is>
       </c>
       <c r="H31" s="18" t="n"/>
@@ -4135,11 +3855,11 @@
     <row r="32">
       <c r="A32" s="15" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P4</t>
         </is>
       </c>
       <c r="B32" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C32" s="15" t="inlineStr">
         <is>
@@ -4148,22 +3868,22 @@
       </c>
       <c r="D32" s="15" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E32" s="15" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="F32" s="15" t="inlineStr">
         <is>
-          <t>Hydrant not there</t>
+          <t>Routine check</t>
         </is>
       </c>
       <c r="G32" s="15" t="inlineStr">
         <is>
-          <t>0718</t>
+          <t>0353</t>
         </is>
       </c>
       <c r="H32" s="18" t="n"/>
@@ -4175,11 +3895,11 @@
     <row r="33">
       <c r="A33" s="15" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P4</t>
         </is>
       </c>
       <c r="B33" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C33" s="15" t="inlineStr">
         <is>
@@ -4188,22 +3908,22 @@
       </c>
       <c r="D33" s="15" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E33" s="15" t="inlineStr">
         <is>
-          <t>T5</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="F33" s="15" t="inlineStr">
         <is>
-          <t>No signal (offline)</t>
+          <t>Low pressure, missing cap</t>
         </is>
       </c>
       <c r="G33" s="15" t="inlineStr">
         <is>
-          <t>3466</t>
+          <t>0564</t>
         </is>
       </c>
       <c r="H33" s="18" t="n"/>
@@ -4215,11 +3935,11 @@
     <row r="34">
       <c r="A34" s="15" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P4</t>
         </is>
       </c>
       <c r="B34" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C34" s="15" t="inlineStr">
         <is>
@@ -4228,22 +3948,22 @@
       </c>
       <c r="D34" s="15" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E34" s="15" t="inlineStr">
         <is>
-          <t>T6</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="F34" s="15" t="inlineStr">
         <is>
-          <t>No account (Survey123 only)</t>
+          <t>Several problems</t>
         </is>
       </c>
       <c r="G34" s="15" t="inlineStr">
         <is>
-          <t>3803</t>
+          <t>3402</t>
         </is>
       </c>
       <c r="H34" s="18" t="n"/>
@@ -4273,17 +3993,17 @@
       </c>
       <c r="E35" s="15" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T4</t>
         </is>
       </c>
       <c r="F35" s="15" t="inlineStr">
         <is>
-          <t>Routine check</t>
+          <t>Hydrant not there</t>
         </is>
       </c>
       <c r="G35" s="15" t="inlineStr">
         <is>
-          <t>0353</t>
+          <t>0570</t>
         </is>
       </c>
       <c r="H35" s="18" t="n"/>
@@ -4313,17 +4033,17 @@
       </c>
       <c r="E36" s="15" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T5</t>
         </is>
       </c>
       <c r="F36" s="15" t="inlineStr">
         <is>
-          <t>Low pressure, missing cap</t>
+          <t>No signal (offline)</t>
         </is>
       </c>
       <c r="G36" s="15" t="inlineStr">
         <is>
-          <t>0564</t>
+          <t>3467</t>
         </is>
       </c>
       <c r="H36" s="18" t="n"/>
@@ -4339,31 +4059,31 @@
         </is>
       </c>
       <c r="B37" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C37" s="15" t="inlineStr">
         <is>
-          <t>Survey123</t>
+          <t>Field Maps</t>
         </is>
       </c>
       <c r="D37" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E37" s="15" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="F37" s="15" t="inlineStr">
         <is>
-          <t>Several problems</t>
+          <t>Routine check</t>
         </is>
       </c>
       <c r="G37" s="15" t="inlineStr">
         <is>
-          <t>3402</t>
+          <t>0291</t>
         </is>
       </c>
       <c r="H37" s="18" t="n"/>
@@ -4379,31 +4099,31 @@
         </is>
       </c>
       <c r="B38" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C38" s="15" t="inlineStr">
         <is>
-          <t>Survey123</t>
+          <t>Field Maps</t>
         </is>
       </c>
       <c r="D38" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E38" s="15" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="F38" s="15" t="inlineStr">
         <is>
-          <t>Hydrant not there</t>
+          <t>Low pressure, missing cap</t>
         </is>
       </c>
       <c r="G38" s="15" t="inlineStr">
         <is>
-          <t>0570</t>
+          <t>0490</t>
         </is>
       </c>
       <c r="H38" s="18" t="n"/>
@@ -4419,31 +4139,31 @@
         </is>
       </c>
       <c r="B39" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C39" s="15" t="inlineStr">
         <is>
-          <t>Survey123</t>
+          <t>Field Maps</t>
         </is>
       </c>
       <c r="D39" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E39" s="15" t="inlineStr">
         <is>
-          <t>T5</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="F39" s="15" t="inlineStr">
         <is>
-          <t>No signal (offline)</t>
+          <t>Several problems</t>
         </is>
       </c>
       <c r="G39" s="15" t="inlineStr">
         <is>
-          <t>3467</t>
+          <t>3641</t>
         </is>
       </c>
       <c r="H39" s="18" t="n"/>
@@ -4459,31 +4179,31 @@
         </is>
       </c>
       <c r="B40" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C40" s="15" t="inlineStr">
         <is>
-          <t>Survey123</t>
+          <t>Field Maps</t>
         </is>
       </c>
       <c r="D40" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E40" s="15" t="inlineStr">
         <is>
-          <t>T6</t>
+          <t>T4</t>
         </is>
       </c>
       <c r="F40" s="15" t="inlineStr">
         <is>
-          <t>No account (Survey123 only)</t>
+          <t>Hydrant not there</t>
         </is>
       </c>
       <c r="G40" s="15" t="inlineStr">
         <is>
-          <t>3808</t>
+          <t>0718</t>
         </is>
       </c>
       <c r="H40" s="18" t="n"/>
@@ -4513,17 +4233,17 @@
       </c>
       <c r="E41" s="15" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T5</t>
         </is>
       </c>
       <c r="F41" s="15" t="inlineStr">
         <is>
-          <t>Routine check</t>
+          <t>No signal (offline)</t>
         </is>
       </c>
       <c r="G41" s="15" t="inlineStr">
         <is>
-          <t>0291</t>
+          <t>3466</t>
         </is>
       </c>
       <c r="H41" s="18" t="n"/>
@@ -4535,11 +4255,11 @@
     <row r="42">
       <c r="A42" s="15" t="inlineStr">
         <is>
-          <t>P4</t>
+          <t>P5</t>
         </is>
       </c>
       <c r="B42" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C42" s="15" t="inlineStr">
         <is>
@@ -4553,17 +4273,17 @@
       </c>
       <c r="E42" s="15" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="F42" s="15" t="inlineStr">
         <is>
-          <t>Low pressure, missing cap</t>
+          <t>Routine check</t>
         </is>
       </c>
       <c r="G42" s="15" t="inlineStr">
         <is>
-          <t>0490</t>
+          <t>0291</t>
         </is>
       </c>
       <c r="H42" s="18" t="n"/>
@@ -4575,11 +4295,11 @@
     <row r="43">
       <c r="A43" s="15" t="inlineStr">
         <is>
-          <t>P4</t>
+          <t>P5</t>
         </is>
       </c>
       <c r="B43" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C43" s="15" t="inlineStr">
         <is>
@@ -4593,17 +4313,17 @@
       </c>
       <c r="E43" s="15" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="F43" s="15" t="inlineStr">
         <is>
-          <t>Several problems</t>
+          <t>Low pressure, missing cap</t>
         </is>
       </c>
       <c r="G43" s="15" t="inlineStr">
         <is>
-          <t>3641</t>
+          <t>0490</t>
         </is>
       </c>
       <c r="H43" s="18" t="n"/>
@@ -4615,11 +4335,11 @@
     <row r="44">
       <c r="A44" s="15" t="inlineStr">
         <is>
-          <t>P4</t>
+          <t>P5</t>
         </is>
       </c>
       <c r="B44" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C44" s="15" t="inlineStr">
         <is>
@@ -4633,17 +4353,17 @@
       </c>
       <c r="E44" s="15" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="F44" s="15" t="inlineStr">
         <is>
-          <t>Hydrant not there</t>
+          <t>Several problems</t>
         </is>
       </c>
       <c r="G44" s="15" t="inlineStr">
         <is>
-          <t>0718</t>
+          <t>3641</t>
         </is>
       </c>
       <c r="H44" s="18" t="n"/>
@@ -4655,11 +4375,11 @@
     <row r="45">
       <c r="A45" s="15" t="inlineStr">
         <is>
-          <t>P4</t>
+          <t>P5</t>
         </is>
       </c>
       <c r="B45" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C45" s="15" t="inlineStr">
         <is>
@@ -4673,17 +4393,17 @@
       </c>
       <c r="E45" s="15" t="inlineStr">
         <is>
-          <t>T5</t>
+          <t>T4</t>
         </is>
       </c>
       <c r="F45" s="15" t="inlineStr">
         <is>
-          <t>No signal (offline)</t>
+          <t>Hydrant not there</t>
         </is>
       </c>
       <c r="G45" s="15" t="inlineStr">
         <is>
-          <t>3466</t>
+          <t>0718</t>
         </is>
       </c>
       <c r="H45" s="18" t="n"/>
@@ -4713,17 +4433,17 @@
       </c>
       <c r="E46" s="15" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T5</t>
         </is>
       </c>
       <c r="F46" s="15" t="inlineStr">
         <is>
-          <t>Routine check</t>
+          <t>No signal (offline)</t>
         </is>
       </c>
       <c r="G46" s="15" t="inlineStr">
         <is>
-          <t>0291</t>
+          <t>3466</t>
         </is>
       </c>
       <c r="H46" s="18" t="n"/>
@@ -4739,31 +4459,31 @@
         </is>
       </c>
       <c r="B47" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C47" s="15" t="inlineStr">
         <is>
-          <t>Field Maps</t>
+          <t>Survey123</t>
         </is>
       </c>
       <c r="D47" s="15" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E47" s="15" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="F47" s="15" t="inlineStr">
         <is>
-          <t>Low pressure, missing cap</t>
+          <t>Routine check</t>
         </is>
       </c>
       <c r="G47" s="15" t="inlineStr">
         <is>
-          <t>0490</t>
+          <t>0353</t>
         </is>
       </c>
       <c r="H47" s="18" t="n"/>
@@ -4779,31 +4499,31 @@
         </is>
       </c>
       <c r="B48" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C48" s="15" t="inlineStr">
         <is>
-          <t>Field Maps</t>
+          <t>Survey123</t>
         </is>
       </c>
       <c r="D48" s="15" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E48" s="15" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="F48" s="15" t="inlineStr">
         <is>
-          <t>Several problems</t>
+          <t>Low pressure, missing cap</t>
         </is>
       </c>
       <c r="G48" s="15" t="inlineStr">
         <is>
-          <t>3641</t>
+          <t>0564</t>
         </is>
       </c>
       <c r="H48" s="18" t="n"/>
@@ -4819,31 +4539,31 @@
         </is>
       </c>
       <c r="B49" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C49" s="15" t="inlineStr">
         <is>
-          <t>Field Maps</t>
+          <t>Survey123</t>
         </is>
       </c>
       <c r="D49" s="15" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E49" s="15" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="F49" s="15" t="inlineStr">
         <is>
-          <t>Hydrant not there</t>
+          <t>Several problems</t>
         </is>
       </c>
       <c r="G49" s="15" t="inlineStr">
         <is>
-          <t>0718</t>
+          <t>3402</t>
         </is>
       </c>
       <c r="H49" s="18" t="n"/>
@@ -4859,31 +4579,31 @@
         </is>
       </c>
       <c r="B50" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C50" s="15" t="inlineStr">
         <is>
-          <t>Field Maps</t>
+          <t>Survey123</t>
         </is>
       </c>
       <c r="D50" s="15" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E50" s="15" t="inlineStr">
         <is>
-          <t>T5</t>
+          <t>T4</t>
         </is>
       </c>
       <c r="F50" s="15" t="inlineStr">
         <is>
-          <t>No signal (offline)</t>
+          <t>Hydrant not there</t>
         </is>
       </c>
       <c r="G50" s="15" t="inlineStr">
         <is>
-          <t>3466</t>
+          <t>0570</t>
         </is>
       </c>
       <c r="H50" s="18" t="n"/>
@@ -4913,17 +4633,17 @@
       </c>
       <c r="E51" s="15" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T5</t>
         </is>
       </c>
       <c r="F51" s="15" t="inlineStr">
         <is>
-          <t>Routine check</t>
+          <t>No signal (offline)</t>
         </is>
       </c>
       <c r="G51" s="15" t="inlineStr">
         <is>
-          <t>0353</t>
+          <t>3467</t>
         </is>
       </c>
       <c r="H51" s="18" t="n"/>
@@ -4935,11 +4655,11 @@
     <row r="52">
       <c r="A52" s="15" t="inlineStr">
         <is>
-          <t>P5</t>
+          <t>P6</t>
         </is>
       </c>
       <c r="B52" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C52" s="15" t="inlineStr">
         <is>
@@ -4948,22 +4668,22 @@
       </c>
       <c r="D52" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E52" s="15" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="F52" s="15" t="inlineStr">
         <is>
-          <t>Low pressure, missing cap</t>
+          <t>Routine check</t>
         </is>
       </c>
       <c r="G52" s="15" t="inlineStr">
         <is>
-          <t>0564</t>
+          <t>0291</t>
         </is>
       </c>
       <c r="H52" s="18" t="n"/>
@@ -4975,11 +4695,11 @@
     <row r="53">
       <c r="A53" s="15" t="inlineStr">
         <is>
-          <t>P5</t>
+          <t>P6</t>
         </is>
       </c>
       <c r="B53" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C53" s="15" t="inlineStr">
         <is>
@@ -4988,22 +4708,22 @@
       </c>
       <c r="D53" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E53" s="15" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="F53" s="15" t="inlineStr">
         <is>
-          <t>Several problems</t>
+          <t>Low pressure, missing cap</t>
         </is>
       </c>
       <c r="G53" s="15" t="inlineStr">
         <is>
-          <t>3402</t>
+          <t>0490</t>
         </is>
       </c>
       <c r="H53" s="18" t="n"/>
@@ -5015,11 +4735,11 @@
     <row r="54">
       <c r="A54" s="15" t="inlineStr">
         <is>
-          <t>P5</t>
+          <t>P6</t>
         </is>
       </c>
       <c r="B54" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C54" s="15" t="inlineStr">
         <is>
@@ -5028,22 +4748,22 @@
       </c>
       <c r="D54" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E54" s="15" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="F54" s="15" t="inlineStr">
         <is>
-          <t>Hydrant not there</t>
+          <t>Several problems</t>
         </is>
       </c>
       <c r="G54" s="15" t="inlineStr">
         <is>
-          <t>0570</t>
+          <t>3641</t>
         </is>
       </c>
       <c r="H54" s="18" t="n"/>
@@ -5055,11 +4775,11 @@
     <row r="55">
       <c r="A55" s="15" t="inlineStr">
         <is>
-          <t>P5</t>
+          <t>P6</t>
         </is>
       </c>
       <c r="B55" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C55" s="15" t="inlineStr">
         <is>
@@ -5068,22 +4788,22 @@
       </c>
       <c r="D55" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E55" s="15" t="inlineStr">
         <is>
-          <t>T5</t>
+          <t>T4</t>
         </is>
       </c>
       <c r="F55" s="15" t="inlineStr">
         <is>
-          <t>No signal (offline)</t>
+          <t>Hydrant not there</t>
         </is>
       </c>
       <c r="G55" s="15" t="inlineStr">
         <is>
-          <t>3467</t>
+          <t>0718</t>
         </is>
       </c>
       <c r="H55" s="18" t="n"/>
@@ -5095,11 +4815,11 @@
     <row r="56">
       <c r="A56" s="15" t="inlineStr">
         <is>
-          <t>P5</t>
+          <t>P6</t>
         </is>
       </c>
       <c r="B56" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C56" s="15" t="inlineStr">
         <is>
@@ -5108,22 +4828,22 @@
       </c>
       <c r="D56" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E56" s="15" t="inlineStr">
         <is>
-          <t>T6</t>
+          <t>T5</t>
         </is>
       </c>
       <c r="F56" s="15" t="inlineStr">
         <is>
-          <t>No account (Survey123 only)</t>
+          <t>No signal (offline)</t>
         </is>
       </c>
       <c r="G56" s="15" t="inlineStr">
         <is>
-          <t>3808</t>
+          <t>3466</t>
         </is>
       </c>
       <c r="H56" s="18" t="n"/>
@@ -5139,16 +4859,16 @@
         </is>
       </c>
       <c r="B57" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C57" s="15" t="inlineStr">
         <is>
-          <t>Survey123</t>
+          <t>Field Maps</t>
         </is>
       </c>
       <c r="D57" s="15" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E57" s="15" t="inlineStr">
@@ -5163,7 +4883,7 @@
       </c>
       <c r="G57" s="15" t="inlineStr">
         <is>
-          <t>0291</t>
+          <t>0353</t>
         </is>
       </c>
       <c r="H57" s="18" t="n"/>
@@ -5179,16 +4899,16 @@
         </is>
       </c>
       <c r="B58" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C58" s="15" t="inlineStr">
         <is>
-          <t>Survey123</t>
+          <t>Field Maps</t>
         </is>
       </c>
       <c r="D58" s="15" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E58" s="15" t="inlineStr">
@@ -5203,7 +4923,7 @@
       </c>
       <c r="G58" s="15" t="inlineStr">
         <is>
-          <t>0490</t>
+          <t>0564</t>
         </is>
       </c>
       <c r="H58" s="18" t="n"/>
@@ -5219,16 +4939,16 @@
         </is>
       </c>
       <c r="B59" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C59" s="15" t="inlineStr">
         <is>
-          <t>Survey123</t>
+          <t>Field Maps</t>
         </is>
       </c>
       <c r="D59" s="15" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E59" s="15" t="inlineStr">
@@ -5243,7 +4963,7 @@
       </c>
       <c r="G59" s="15" t="inlineStr">
         <is>
-          <t>3641</t>
+          <t>3402</t>
         </is>
       </c>
       <c r="H59" s="18" t="n"/>
@@ -5259,16 +4979,16 @@
         </is>
       </c>
       <c r="B60" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C60" s="15" t="inlineStr">
         <is>
-          <t>Survey123</t>
+          <t>Field Maps</t>
         </is>
       </c>
       <c r="D60" s="15" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E60" s="15" t="inlineStr">
@@ -5283,7 +5003,7 @@
       </c>
       <c r="G60" s="15" t="inlineStr">
         <is>
-          <t>0718</t>
+          <t>0570</t>
         </is>
       </c>
       <c r="H60" s="18" t="n"/>
@@ -5299,16 +5019,16 @@
         </is>
       </c>
       <c r="B61" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C61" s="15" t="inlineStr">
         <is>
-          <t>Survey123</t>
+          <t>Field Maps</t>
         </is>
       </c>
       <c r="D61" s="15" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E61" s="15" t="inlineStr">
@@ -5323,7 +5043,7 @@
       </c>
       <c r="G61" s="15" t="inlineStr">
         <is>
-          <t>3466</t>
+          <t>3467</t>
         </is>
       </c>
       <c r="H61" s="18" t="n"/>
@@ -5335,7 +5055,7 @@
     <row r="62">
       <c r="A62" s="15" t="inlineStr">
         <is>
-          <t>P6</t>
+          <t>P7</t>
         </is>
       </c>
       <c r="B62" s="15" t="n">
@@ -5343,27 +5063,27 @@
       </c>
       <c r="C62" s="15" t="inlineStr">
         <is>
-          <t>Survey123</t>
+          <t>Field Maps</t>
         </is>
       </c>
       <c r="D62" s="15" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E62" s="15" t="inlineStr">
         <is>
-          <t>T6</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="F62" s="15" t="inlineStr">
         <is>
-          <t>No account (Survey123 only)</t>
+          <t>Routine check</t>
         </is>
       </c>
       <c r="G62" s="15" t="inlineStr">
         <is>
-          <t>3803</t>
+          <t>0353</t>
         </is>
       </c>
       <c r="H62" s="18" t="n"/>
@@ -5375,11 +5095,11 @@
     <row r="63">
       <c r="A63" s="15" t="inlineStr">
         <is>
-          <t>P6</t>
+          <t>P7</t>
         </is>
       </c>
       <c r="B63" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C63" s="15" t="inlineStr">
         <is>
@@ -5393,17 +5113,17 @@
       </c>
       <c r="E63" s="15" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="F63" s="15" t="inlineStr">
         <is>
-          <t>Routine check</t>
+          <t>Low pressure, missing cap</t>
         </is>
       </c>
       <c r="G63" s="15" t="inlineStr">
         <is>
-          <t>0353</t>
+          <t>0564</t>
         </is>
       </c>
       <c r="H63" s="18" t="n"/>
@@ -5415,11 +5135,11 @@
     <row r="64">
       <c r="A64" s="15" t="inlineStr">
         <is>
-          <t>P6</t>
+          <t>P7</t>
         </is>
       </c>
       <c r="B64" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C64" s="15" t="inlineStr">
         <is>
@@ -5433,17 +5153,17 @@
       </c>
       <c r="E64" s="15" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="F64" s="15" t="inlineStr">
         <is>
-          <t>Low pressure, missing cap</t>
+          <t>Several problems</t>
         </is>
       </c>
       <c r="G64" s="15" t="inlineStr">
         <is>
-          <t>0564</t>
+          <t>3402</t>
         </is>
       </c>
       <c r="H64" s="18" t="n"/>
@@ -5455,11 +5175,11 @@
     <row r="65">
       <c r="A65" s="15" t="inlineStr">
         <is>
-          <t>P6</t>
+          <t>P7</t>
         </is>
       </c>
       <c r="B65" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C65" s="15" t="inlineStr">
         <is>
@@ -5473,17 +5193,17 @@
       </c>
       <c r="E65" s="15" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T4</t>
         </is>
       </c>
       <c r="F65" s="15" t="inlineStr">
         <is>
-          <t>Several problems</t>
+          <t>Hydrant not there</t>
         </is>
       </c>
       <c r="G65" s="15" t="inlineStr">
         <is>
-          <t>3402</t>
+          <t>0570</t>
         </is>
       </c>
       <c r="H65" s="18" t="n"/>
@@ -5495,11 +5215,11 @@
     <row r="66">
       <c r="A66" s="15" t="inlineStr">
         <is>
-          <t>P6</t>
+          <t>P7</t>
         </is>
       </c>
       <c r="B66" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C66" s="15" t="inlineStr">
         <is>
@@ -5513,17 +5233,17 @@
       </c>
       <c r="E66" s="15" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>T5</t>
         </is>
       </c>
       <c r="F66" s="15" t="inlineStr">
         <is>
-          <t>Hydrant not there</t>
+          <t>No signal (offline)</t>
         </is>
       </c>
       <c r="G66" s="15" t="inlineStr">
         <is>
-          <t>0570</t>
+          <t>3467</t>
         </is>
       </c>
       <c r="H66" s="18" t="n"/>
@@ -5535,7 +5255,7 @@
     <row r="67">
       <c r="A67" s="15" t="inlineStr">
         <is>
-          <t>P6</t>
+          <t>P7</t>
         </is>
       </c>
       <c r="B67" s="15" t="n">
@@ -5543,27 +5263,27 @@
       </c>
       <c r="C67" s="15" t="inlineStr">
         <is>
-          <t>Field Maps</t>
+          <t>Survey123</t>
         </is>
       </c>
       <c r="D67" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E67" s="15" t="inlineStr">
         <is>
-          <t>T5</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="F67" s="15" t="inlineStr">
         <is>
-          <t>No signal (offline)</t>
+          <t>Routine check</t>
         </is>
       </c>
       <c r="G67" s="15" t="inlineStr">
         <is>
-          <t>3467</t>
+          <t>0291</t>
         </is>
       </c>
       <c r="H67" s="18" t="n"/>
@@ -5579,31 +5299,31 @@
         </is>
       </c>
       <c r="B68" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C68" s="15" t="inlineStr">
         <is>
-          <t>Field Maps</t>
+          <t>Survey123</t>
         </is>
       </c>
       <c r="D68" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E68" s="15" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="F68" s="15" t="inlineStr">
         <is>
-          <t>Routine check</t>
+          <t>Low pressure, missing cap</t>
         </is>
       </c>
       <c r="G68" s="15" t="inlineStr">
         <is>
-          <t>0353</t>
+          <t>0490</t>
         </is>
       </c>
       <c r="H68" s="18" t="n"/>
@@ -5619,31 +5339,31 @@
         </is>
       </c>
       <c r="B69" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C69" s="15" t="inlineStr">
         <is>
-          <t>Field Maps</t>
+          <t>Survey123</t>
         </is>
       </c>
       <c r="D69" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E69" s="15" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="F69" s="15" t="inlineStr">
         <is>
-          <t>Low pressure, missing cap</t>
+          <t>Several problems</t>
         </is>
       </c>
       <c r="G69" s="15" t="inlineStr">
         <is>
-          <t>0564</t>
+          <t>3641</t>
         </is>
       </c>
       <c r="H69" s="18" t="n"/>
@@ -5659,31 +5379,31 @@
         </is>
       </c>
       <c r="B70" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C70" s="15" t="inlineStr">
         <is>
-          <t>Field Maps</t>
+          <t>Survey123</t>
         </is>
       </c>
       <c r="D70" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E70" s="15" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T4</t>
         </is>
       </c>
       <c r="F70" s="15" t="inlineStr">
         <is>
-          <t>Several problems</t>
+          <t>Hydrant not there</t>
         </is>
       </c>
       <c r="G70" s="15" t="inlineStr">
         <is>
-          <t>3402</t>
+          <t>0718</t>
         </is>
       </c>
       <c r="H70" s="18" t="n"/>
@@ -5699,31 +5419,31 @@
         </is>
       </c>
       <c r="B71" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C71" s="15" t="inlineStr">
         <is>
-          <t>Field Maps</t>
+          <t>Survey123</t>
         </is>
       </c>
       <c r="D71" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E71" s="15" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>T5</t>
         </is>
       </c>
       <c r="F71" s="15" t="inlineStr">
         <is>
-          <t>Hydrant not there</t>
+          <t>No signal (offline)</t>
         </is>
       </c>
       <c r="G71" s="15" t="inlineStr">
         <is>
-          <t>0570</t>
+          <t>3466</t>
         </is>
       </c>
       <c r="H71" s="18" t="n"/>
@@ -5735,7 +5455,7 @@
     <row r="72">
       <c r="A72" s="15" t="inlineStr">
         <is>
-          <t>P7</t>
+          <t>P8</t>
         </is>
       </c>
       <c r="B72" s="15" t="n">
@@ -5743,7 +5463,7 @@
       </c>
       <c r="C72" s="15" t="inlineStr">
         <is>
-          <t>Field Maps</t>
+          <t>Survey123</t>
         </is>
       </c>
       <c r="D72" s="15" t="inlineStr">
@@ -5753,17 +5473,17 @@
       </c>
       <c r="E72" s="15" t="inlineStr">
         <is>
-          <t>T5</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="F72" s="15" t="inlineStr">
         <is>
-          <t>No signal (offline)</t>
+          <t>Routine check</t>
         </is>
       </c>
       <c r="G72" s="15" t="inlineStr">
         <is>
-          <t>3467</t>
+          <t>0353</t>
         </is>
       </c>
       <c r="H72" s="18" t="n"/>
@@ -5775,11 +5495,11 @@
     <row r="73">
       <c r="A73" s="15" t="inlineStr">
         <is>
-          <t>P7</t>
+          <t>P8</t>
         </is>
       </c>
       <c r="B73" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C73" s="15" t="inlineStr">
         <is>
@@ -5788,22 +5508,22 @@
       </c>
       <c r="D73" s="15" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E73" s="15" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="F73" s="15" t="inlineStr">
         <is>
-          <t>Routine check</t>
+          <t>Low pressure, missing cap</t>
         </is>
       </c>
       <c r="G73" s="15" t="inlineStr">
         <is>
-          <t>0291</t>
+          <t>0564</t>
         </is>
       </c>
       <c r="H73" s="18" t="n"/>
@@ -5815,11 +5535,11 @@
     <row r="74">
       <c r="A74" s="15" t="inlineStr">
         <is>
-          <t>P7</t>
+          <t>P8</t>
         </is>
       </c>
       <c r="B74" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C74" s="15" t="inlineStr">
         <is>
@@ -5828,22 +5548,22 @@
       </c>
       <c r="D74" s="15" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E74" s="15" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="F74" s="15" t="inlineStr">
         <is>
-          <t>Low pressure, missing cap</t>
+          <t>Several problems</t>
         </is>
       </c>
       <c r="G74" s="15" t="inlineStr">
         <is>
-          <t>0490</t>
+          <t>3402</t>
         </is>
       </c>
       <c r="H74" s="18" t="n"/>
@@ -5855,11 +5575,11 @@
     <row r="75">
       <c r="A75" s="15" t="inlineStr">
         <is>
-          <t>P7</t>
+          <t>P8</t>
         </is>
       </c>
       <c r="B75" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C75" s="15" t="inlineStr">
         <is>
@@ -5868,22 +5588,22 @@
       </c>
       <c r="D75" s="15" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E75" s="15" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T4</t>
         </is>
       </c>
       <c r="F75" s="15" t="inlineStr">
         <is>
-          <t>Several problems</t>
+          <t>Hydrant not there</t>
         </is>
       </c>
       <c r="G75" s="15" t="inlineStr">
         <is>
-          <t>3641</t>
+          <t>0570</t>
         </is>
       </c>
       <c r="H75" s="18" t="n"/>
@@ -5895,11 +5615,11 @@
     <row r="76">
       <c r="A76" s="15" t="inlineStr">
         <is>
-          <t>P7</t>
+          <t>P8</t>
         </is>
       </c>
       <c r="B76" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C76" s="15" t="inlineStr">
         <is>
@@ -5908,22 +5628,22 @@
       </c>
       <c r="D76" s="15" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E76" s="15" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>T5</t>
         </is>
       </c>
       <c r="F76" s="15" t="inlineStr">
         <is>
-          <t>Hydrant not there</t>
+          <t>No signal (offline)</t>
         </is>
       </c>
       <c r="G76" s="15" t="inlineStr">
         <is>
-          <t>0718</t>
+          <t>3467</t>
         </is>
       </c>
       <c r="H76" s="18" t="n"/>
@@ -5935,7 +5655,7 @@
     <row r="77">
       <c r="A77" s="15" t="inlineStr">
         <is>
-          <t>P7</t>
+          <t>P8</t>
         </is>
       </c>
       <c r="B77" s="15" t="n">
@@ -5943,7 +5663,7 @@
       </c>
       <c r="C77" s="15" t="inlineStr">
         <is>
-          <t>Survey123</t>
+          <t>Field Maps</t>
         </is>
       </c>
       <c r="D77" s="15" t="inlineStr">
@@ -5953,17 +5673,17 @@
       </c>
       <c r="E77" s="15" t="inlineStr">
         <is>
-          <t>T5</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="F77" s="15" t="inlineStr">
         <is>
-          <t>No signal (offline)</t>
+          <t>Routine check</t>
         </is>
       </c>
       <c r="G77" s="15" t="inlineStr">
         <is>
-          <t>3466</t>
+          <t>0291</t>
         </is>
       </c>
       <c r="H77" s="18" t="n"/>
@@ -5975,7 +5695,7 @@
     <row r="78">
       <c r="A78" s="15" t="inlineStr">
         <is>
-          <t>P7</t>
+          <t>P8</t>
         </is>
       </c>
       <c r="B78" s="15" t="n">
@@ -5983,7 +5703,7 @@
       </c>
       <c r="C78" s="15" t="inlineStr">
         <is>
-          <t>Survey123</t>
+          <t>Field Maps</t>
         </is>
       </c>
       <c r="D78" s="15" t="inlineStr">
@@ -5993,17 +5713,17 @@
       </c>
       <c r="E78" s="15" t="inlineStr">
         <is>
-          <t>T6</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="F78" s="15" t="inlineStr">
         <is>
-          <t>No account (Survey123 only)</t>
+          <t>Low pressure, missing cap</t>
         </is>
       </c>
       <c r="G78" s="15" t="inlineStr">
         <is>
-          <t>3803</t>
+          <t>0490</t>
         </is>
       </c>
       <c r="H78" s="18" t="n"/>
@@ -6019,31 +5739,31 @@
         </is>
       </c>
       <c r="B79" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C79" s="15" t="inlineStr">
         <is>
-          <t>Survey123</t>
+          <t>Field Maps</t>
         </is>
       </c>
       <c r="D79" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E79" s="15" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="F79" s="15" t="inlineStr">
         <is>
-          <t>Routine check</t>
+          <t>Several problems</t>
         </is>
       </c>
       <c r="G79" s="15" t="inlineStr">
         <is>
-          <t>0353</t>
+          <t>3641</t>
         </is>
       </c>
       <c r="H79" s="18" t="n"/>
@@ -6059,31 +5779,31 @@
         </is>
       </c>
       <c r="B80" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C80" s="15" t="inlineStr">
         <is>
-          <t>Survey123</t>
+          <t>Field Maps</t>
         </is>
       </c>
       <c r="D80" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E80" s="15" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T4</t>
         </is>
       </c>
       <c r="F80" s="15" t="inlineStr">
         <is>
-          <t>Low pressure, missing cap</t>
+          <t>Hydrant not there</t>
         </is>
       </c>
       <c r="G80" s="15" t="inlineStr">
         <is>
-          <t>0564</t>
+          <t>0718</t>
         </is>
       </c>
       <c r="H80" s="18" t="n"/>
@@ -6099,31 +5819,31 @@
         </is>
       </c>
       <c r="B81" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C81" s="15" t="inlineStr">
         <is>
-          <t>Survey123</t>
+          <t>Field Maps</t>
         </is>
       </c>
       <c r="D81" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E81" s="15" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T5</t>
         </is>
       </c>
       <c r="F81" s="15" t="inlineStr">
         <is>
-          <t>Several problems</t>
+          <t>No signal (offline)</t>
         </is>
       </c>
       <c r="G81" s="15" t="inlineStr">
         <is>
-          <t>3402</t>
+          <t>3466</t>
         </is>
       </c>
       <c r="H81" s="18" t="n"/>
@@ -6132,339 +5852,19 @@
       <c r="K81" s="16" t="n"/>
       <c r="L81" s="16" t="n"/>
     </row>
-    <row r="82">
-      <c r="A82" s="15" t="inlineStr">
-        <is>
-          <t>P8</t>
-        </is>
-      </c>
-      <c r="B82" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="C82" s="15" t="inlineStr">
-        <is>
-          <t>Survey123</t>
-        </is>
-      </c>
-      <c r="D82" s="15" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="E82" s="15" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="F82" s="15" t="inlineStr">
-        <is>
-          <t>Hydrant not there</t>
-        </is>
-      </c>
-      <c r="G82" s="15" t="inlineStr">
-        <is>
-          <t>0570</t>
-        </is>
-      </c>
-      <c r="H82" s="18" t="n"/>
-      <c r="I82" s="16" t="n"/>
-      <c r="J82" s="16" t="n"/>
-      <c r="K82" s="16" t="n"/>
-      <c r="L82" s="16" t="n"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="15" t="inlineStr">
-        <is>
-          <t>P8</t>
-        </is>
-      </c>
-      <c r="B83" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="C83" s="15" t="inlineStr">
-        <is>
-          <t>Survey123</t>
-        </is>
-      </c>
-      <c r="D83" s="15" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="E83" s="15" t="inlineStr">
-        <is>
-          <t>T5</t>
-        </is>
-      </c>
-      <c r="F83" s="15" t="inlineStr">
-        <is>
-          <t>No signal (offline)</t>
-        </is>
-      </c>
-      <c r="G83" s="15" t="inlineStr">
-        <is>
-          <t>3467</t>
-        </is>
-      </c>
-      <c r="H83" s="18" t="n"/>
-      <c r="I83" s="16" t="n"/>
-      <c r="J83" s="16" t="n"/>
-      <c r="K83" s="16" t="n"/>
-      <c r="L83" s="16" t="n"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="15" t="inlineStr">
-        <is>
-          <t>P8</t>
-        </is>
-      </c>
-      <c r="B84" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="C84" s="15" t="inlineStr">
-        <is>
-          <t>Survey123</t>
-        </is>
-      </c>
-      <c r="D84" s="15" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="E84" s="15" t="inlineStr">
-        <is>
-          <t>T6</t>
-        </is>
-      </c>
-      <c r="F84" s="15" t="inlineStr">
-        <is>
-          <t>No account (Survey123 only)</t>
-        </is>
-      </c>
-      <c r="G84" s="15" t="inlineStr">
-        <is>
-          <t>3808</t>
-        </is>
-      </c>
-      <c r="H84" s="18" t="n"/>
-      <c r="I84" s="16" t="n"/>
-      <c r="J84" s="16" t="n"/>
-      <c r="K84" s="16" t="n"/>
-      <c r="L84" s="16" t="n"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="15" t="inlineStr">
-        <is>
-          <t>P8</t>
-        </is>
-      </c>
-      <c r="B85" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="C85" s="15" t="inlineStr">
-        <is>
-          <t>Field Maps</t>
-        </is>
-      </c>
-      <c r="D85" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E85" s="15" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="F85" s="15" t="inlineStr">
-        <is>
-          <t>Routine check</t>
-        </is>
-      </c>
-      <c r="G85" s="15" t="inlineStr">
-        <is>
-          <t>0291</t>
-        </is>
-      </c>
-      <c r="H85" s="18" t="n"/>
-      <c r="I85" s="16" t="n"/>
-      <c r="J85" s="16" t="n"/>
-      <c r="K85" s="16" t="n"/>
-      <c r="L85" s="16" t="n"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="15" t="inlineStr">
-        <is>
-          <t>P8</t>
-        </is>
-      </c>
-      <c r="B86" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="C86" s="15" t="inlineStr">
-        <is>
-          <t>Field Maps</t>
-        </is>
-      </c>
-      <c r="D86" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E86" s="15" t="inlineStr">
-        <is>
-          <t>T2</t>
-        </is>
-      </c>
-      <c r="F86" s="15" t="inlineStr">
-        <is>
-          <t>Low pressure, missing cap</t>
-        </is>
-      </c>
-      <c r="G86" s="15" t="inlineStr">
-        <is>
-          <t>0490</t>
-        </is>
-      </c>
-      <c r="H86" s="18" t="n"/>
-      <c r="I86" s="16" t="n"/>
-      <c r="J86" s="16" t="n"/>
-      <c r="K86" s="16" t="n"/>
-      <c r="L86" s="16" t="n"/>
-    </row>
-    <row r="87">
-      <c r="A87" s="15" t="inlineStr">
-        <is>
-          <t>P8</t>
-        </is>
-      </c>
-      <c r="B87" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="C87" s="15" t="inlineStr">
-        <is>
-          <t>Field Maps</t>
-        </is>
-      </c>
-      <c r="D87" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E87" s="15" t="inlineStr">
-        <is>
-          <t>T3</t>
-        </is>
-      </c>
-      <c r="F87" s="15" t="inlineStr">
-        <is>
-          <t>Several problems</t>
-        </is>
-      </c>
-      <c r="G87" s="15" t="inlineStr">
-        <is>
-          <t>3641</t>
-        </is>
-      </c>
-      <c r="H87" s="18" t="n"/>
-      <c r="I87" s="16" t="n"/>
-      <c r="J87" s="16" t="n"/>
-      <c r="K87" s="16" t="n"/>
-      <c r="L87" s="16" t="n"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="15" t="inlineStr">
-        <is>
-          <t>P8</t>
-        </is>
-      </c>
-      <c r="B88" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="C88" s="15" t="inlineStr">
-        <is>
-          <t>Field Maps</t>
-        </is>
-      </c>
-      <c r="D88" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E88" s="15" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="F88" s="15" t="inlineStr">
-        <is>
-          <t>Hydrant not there</t>
-        </is>
-      </c>
-      <c r="G88" s="15" t="inlineStr">
-        <is>
-          <t>0718</t>
-        </is>
-      </c>
-      <c r="H88" s="18" t="n"/>
-      <c r="I88" s="16" t="n"/>
-      <c r="J88" s="16" t="n"/>
-      <c r="K88" s="16" t="n"/>
-      <c r="L88" s="16" t="n"/>
-    </row>
-    <row r="89">
-      <c r="A89" s="15" t="inlineStr">
-        <is>
-          <t>P8</t>
-        </is>
-      </c>
-      <c r="B89" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="C89" s="15" t="inlineStr">
-        <is>
-          <t>Field Maps</t>
-        </is>
-      </c>
-      <c r="D89" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E89" s="15" t="inlineStr">
-        <is>
-          <t>T5</t>
-        </is>
-      </c>
-      <c r="F89" s="15" t="inlineStr">
-        <is>
-          <t>No signal (offline)</t>
-        </is>
-      </c>
-      <c r="G89" s="15" t="inlineStr">
-        <is>
-          <t>3466</t>
-        </is>
-      </c>
-      <c r="H89" s="18" t="n"/>
-      <c r="I89" s="16" t="n"/>
-      <c r="J89" s="16" t="n"/>
-      <c r="K89" s="16" t="n"/>
-      <c r="L89" s="16" t="n"/>
-    </row>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation sqref="I2:I89" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Alone,With help,Failed,Skipped"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J89" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Enter a whole number from 1 to 7" type="whole" operator="between">
+    <dataValidation sqref="J2:J81" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Enter a whole number from 1 to 7" type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>7</formula2>
     </dataValidation>
-    <dataValidation sqref="K2:K89" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No,Not needed"</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H89" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="decimal" operator="between">
+    <dataValidation sqref="H2:H81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="decimal" operator="between">
       <formula1>0</formula1>
       <formula2>60</formula2>
     </dataValidation>
@@ -8390,7 +7790,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -8448,16 +7848,16 @@
     <row r="2">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>Crews without accounts can inspect</t>
+          <t>Account and licensing cost</t>
         </is>
       </c>
       <c r="B2" s="15" t="inlineStr">
         <is>
-          <t>Any crew member can submit, no sign-in or account request needed</t>
+          <t>No added licenses for 44 engine companies</t>
         </is>
       </c>
       <c r="C2" s="16" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="D2" s="16" t="n"/>
       <c r="E2" s="16" t="n"/>
@@ -8474,16 +7874,16 @@
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
-          <t>Account and licensing cost</t>
+          <t>Inspections tied to the right hydrant</t>
         </is>
       </c>
       <c r="B3" s="15" t="inlineStr">
         <is>
-          <t>No added licenses for 44 engine companies</t>
+          <t>Every record lands under its hydrant without cleanup</t>
         </is>
       </c>
       <c r="C3" s="16" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D3" s="16" t="n"/>
       <c r="E3" s="16" t="n"/>
@@ -8500,12 +7900,12 @@
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
         <is>
-          <t>Inspections tied to the right hydrant</t>
+          <t>Offline</t>
         </is>
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>Every record lands under its hydrant without cleanup</t>
+          <t>Works with no signal, map included, syncs without fuss</t>
         </is>
       </c>
       <c r="C4" s="16" t="n">
@@ -8526,12 +7926,12 @@
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Upkeep</t>
         </is>
       </c>
       <c r="B5" s="15" t="inlineStr">
         <is>
-          <t>Works with no signal, map included, syncs without fuss</t>
+          <t>Form and inspector list are quick to change and roll out</t>
         </is>
       </c>
       <c r="C5" s="16" t="n">
@@ -8552,12 +7952,12 @@
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
         <is>
-          <t>Upkeep</t>
+          <t>Dashboard and annual report</t>
         </is>
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Form and inspector list are quick to change and roll out</t>
+          <t>Dashboard and FY report come straight from the data</t>
         </is>
       </c>
       <c r="C6" s="16" t="n">
@@ -8578,12 +7978,12 @@
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
         <is>
-          <t>Dashboard and annual report</t>
+          <t>Later Maximo link (FME Flow)</t>
         </is>
       </c>
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>Dashboard and FY report come straight from the data</t>
+          <t>Follow-up flags can become work requests with no rework</t>
         </is>
       </c>
       <c r="C7" s="16" t="n">
@@ -8604,12 +8004,12 @@
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
         <is>
-          <t>Later Maximo link (FME Flow)</t>
+          <t>Security and sharing</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>Follow-up flags can become work requests with no rework</t>
+          <t>Fits SFPUC portal policy with no exceptions</t>
         </is>
       </c>
       <c r="C8" s="16" t="n">
@@ -8628,57 +8028,31 @@
       <c r="H8" s="16" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr">
-        <is>
-          <t>Security and sharing</t>
-        </is>
-      </c>
-      <c r="B9" s="15" t="inlineStr">
-        <is>
-          <t>Fits SFPUC portal policy with no exceptions</t>
-        </is>
-      </c>
-      <c r="C9" s="16" t="n">
-        <v>5</v>
-      </c>
-      <c r="D9" s="16" t="n"/>
-      <c r="E9" s="16" t="n"/>
-      <c r="F9" s="15">
-        <f>IF(D9="","",C9*D9)</f>
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="n"/>
+      <c r="C9" s="21">
+        <f>SUM(C2:C8)</f>
         <v/>
       </c>
-      <c r="G9" s="15">
-        <f>IF(E9="","",C9*E9)</f>
+      <c r="D9" s="21" t="n"/>
+      <c r="E9" s="21" t="n"/>
+      <c r="F9" s="20">
+        <f>SUM(F2:F8)</f>
         <v/>
       </c>
-      <c r="H9" s="16" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="20" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B10" s="20" t="n"/>
-      <c r="C10" s="21">
-        <f>SUM(C2:C9)</f>
+      <c r="G9" s="20">
+        <f>SUM(G2:G8)</f>
         <v/>
       </c>
-      <c r="D10" s="21" t="n"/>
-      <c r="E10" s="21" t="n"/>
-      <c r="F10" s="20">
-        <f>SUM(F2:F9)</f>
-        <v/>
-      </c>
-      <c r="G10" s="20">
-        <f>SUM(G2:G9)</f>
-        <v/>
-      </c>
-      <c r="H10" s="21" t="n"/>
+      <c r="H9" s="21" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="D2:E9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Enter a whole number from 1 to 5" type="whole" operator="between">
+    <dataValidation sqref="D2:E8" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Enter a whole number from 1 to 5" type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
@@ -8693,7 +8067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8825,29 +8199,15 @@
       <c r="G8" s="16" t="n"/>
       <c r="H8" s="16" t="n"/>
     </row>
-    <row r="9" ht="60" customHeight="1">
-      <c r="A9" s="15" t="inlineStr">
-        <is>
-          <t>T6 (S123)</t>
-        </is>
-      </c>
-      <c r="B9" s="16" t="n"/>
-      <c r="C9" s="16" t="n"/>
-      <c r="D9" s="16" t="n"/>
-      <c r="E9" s="16" t="n"/>
-      <c r="F9" s="16" t="n"/>
-      <c r="G9" s="16" t="n"/>
-      <c r="H9" s="16" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="23" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="23" t="inlineStr">
         <is>
           <t>After-app (1-5):  Q1 without help ___   Q2 quick enough ___   Q3 one-handed/outdoors ___   Q4 trust it saved ___</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="23" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="23" t="inlineStr">
         <is>
           <t>Most frustrating part:</t>
         </is>

</xml_diff>